<commit_message>
feat: Implement security paper code reset functionality
- Added a modal for resetting security paper codes with reasons for reset.
- Introduced a new service, SecurityPaperCodeService, to handle logic for releasing security paper codes.
- Updated routes to include endpoints for resetting and assigning security paper codes.
- Modified views to integrate the new reset functionality across various modules (Land RofO, SLTR RofO).
- Enhanced database schema to support void status and reasons for security paper code resets.
- Implemented caching logic to ensure availability of security paper codes after reset.
</commit_message>
<xml_diff>
--- a/docs/data/shalf_racks/FileNo Combination_2_Rack C.xlsx
+++ b/docs/data/shalf_racks/FileNo Combination_2_Rack C.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="9302"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="14940" windowHeight="9225" activeTab="0"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
   <si>
     <t>SN</t>
   </si>
@@ -110,43 +110,56 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
   <fonts count="5">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="18"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="18"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -168,349 +181,266 @@
     </border>
     <border>
       <left style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="medium">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment/>
-      <protection/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="6" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
-      <alignment/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="12" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="13" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
-      <alignment/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="14" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="3" builtinId="7"/>
-    <cellStyle name="Comma" xfId="4" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="5" builtinId="6"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <dxfs count="0"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -557,7 +487,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -609,7 +539,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -670,151 +600,185 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50609AE5-2D6D-429A-8726-ABD62466BAA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:R55"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="6" max="6" width="29" customWidth="true" style="0"/>
+    <col min="7" max="7" width="18.85546875" customWidth="true" style="0"/>
+    <col min="16" max="16" width="12.85546875" customWidth="true" style="0"/>
+    <col min="17" max="17" width="22.5703125" customWidth="true" style="0"/>
+    <col min="18" max="18" width="23" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="12.75" thickBot="1">
+    <row r="1" spans="1:18" customHeight="1" ht="24">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -837,7 +801,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="12.75">
+    <row r="2" spans="1:18" customHeight="1" ht="23.25">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -861,7 +825,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="12.75">
+    <row r="3" spans="1:18" customHeight="1" ht="23.25">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -885,7 +849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="12.75">
+    <row r="4" spans="1:18" customHeight="1" ht="23.25">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -909,7 +873,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="12.75">
+    <row r="5" spans="1:18" customHeight="1" ht="23.25">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -933,7 +897,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="12.75">
+    <row r="6" spans="1:18" customHeight="1" ht="23.25">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -957,7 +921,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="12.75">
+    <row r="7" spans="1:18" customHeight="1" ht="23.25">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -981,7 +945,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="12.75">
+    <row r="8" spans="1:18" customHeight="1" ht="23.25">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -1005,7 +969,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="12.75">
+    <row r="9" spans="1:18" customHeight="1" ht="23.25">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -1029,7 +993,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="12.75" thickBot="1">
+    <row r="10" spans="1:18" customHeight="1" ht="24">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -1058,7 +1022,7 @@
         <v>5200</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="12.75">
+    <row r="11" spans="1:18" customHeight="1" ht="23.25">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1087,7 +1051,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="12.75">
+    <row r="12" spans="1:18" customHeight="1" ht="23.25">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -1116,7 +1080,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="12.75">
+    <row r="13" spans="1:18" customHeight="1" ht="23.25">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -1146,7 +1110,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="12.75">
+    <row r="14" spans="1:18" customHeight="1" ht="23.25">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -1170,7 +1134,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="12.75" thickBot="1">
+    <row r="15" spans="1:18" customHeight="1" ht="24">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -1194,7 +1158,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="12.75">
+    <row r="16" spans="1:18" customHeight="1" ht="23.25">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -1218,7 +1182,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="12.75">
+    <row r="17" spans="1:18" customHeight="1" ht="23.25">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -1242,7 +1206,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="12.75">
+    <row r="18" spans="1:18" customHeight="1" ht="23.25">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -1266,7 +1230,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="12.75">
+    <row r="19" spans="1:18" customHeight="1" ht="23.25">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -1290,7 +1254,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="12.75">
+    <row r="20" spans="1:18" customHeight="1" ht="23.25">
       <c r="A20" s="9">
         <v>19</v>
       </c>
@@ -1314,7 +1278,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="12.75">
+    <row r="21" spans="1:18" customHeight="1" ht="23.25">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -1338,7 +1302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="12.75">
+    <row r="22" spans="1:18" customHeight="1" ht="23.25">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -1362,7 +1326,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="12.75">
+    <row r="23" spans="1:18" customHeight="1" ht="23.25">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -1386,7 +1350,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="12.75">
+    <row r="24" spans="1:18" customHeight="1" ht="23.25">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -1410,7 +1374,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="12.75">
+    <row r="25" spans="1:18" customHeight="1" ht="23.25">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -1434,7 +1398,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="12.75">
+    <row r="26" spans="1:18" customHeight="1" ht="23.25">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -1458,7 +1422,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="12.75">
+    <row r="27" spans="1:18" customHeight="1" ht="23.25">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -1482,7 +1446,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="12.75">
+    <row r="28" spans="1:18" customHeight="1" ht="23.25">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -1506,7 +1470,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="12.75" thickBot="1">
+    <row r="29" spans="1:18" customHeight="1" ht="24">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -1530,15 +1494,29 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="12.75">
-      <c r="A30" s="1"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="1"/>
+    <row r="30" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="17">
+        <v>2</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="18">
+        <v>29</v>
+      </c>
+      <c r="E30" s="18" t="str">
+        <f>C30&amp;D30</f>
+        <v>C29</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>9</v>
+      </c>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -1550,15 +1528,29 @@
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
     </row>
-    <row r="31" spans="1:18" ht="12.75">
-      <c r="A31" s="1"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="1"/>
+    <row r="31" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="17">
+        <v>2</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="18">
+        <v>30</v>
+      </c>
+      <c r="E31" s="18" t="str">
+        <f>C31&amp;D31</f>
+        <v>C30</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>10</v>
+      </c>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
@@ -1570,15 +1562,29 @@
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
     </row>
-    <row r="32" spans="1:18" ht="12.75">
-      <c r="A32" s="1"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="1"/>
+    <row r="32" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="17">
+        <v>2</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="18">
+        <v>31</v>
+      </c>
+      <c r="E32" s="18" t="str">
+        <f>C32&amp;D32</f>
+        <v>C31</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>11</v>
+      </c>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -1590,15 +1596,29 @@
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
     </row>
-    <row r="33" spans="1:18" ht="12.75">
-      <c r="A33" s="1"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="1"/>
+    <row r="33" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33" s="17">
+        <v>2</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="18">
+        <v>32</v>
+      </c>
+      <c r="E33" s="18" t="str">
+        <f>C33&amp;D33</f>
+        <v>C32</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>12</v>
+      </c>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
@@ -1610,15 +1630,29 @@
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
     </row>
-    <row r="34" spans="1:18" ht="12.75">
-      <c r="A34" s="1"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="1"/>
+    <row r="34" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="17">
+        <v>2</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="18">
+        <v>33</v>
+      </c>
+      <c r="E34" s="18" t="str">
+        <f>C34&amp;D34</f>
+        <v>C33</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>19</v>
+      </c>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
@@ -1630,15 +1664,29 @@
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
     </row>
-    <row r="35" spans="1:18" ht="12.75">
-      <c r="A35" s="1"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="1"/>
+    <row r="35" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="17">
+        <v>2</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="18">
+        <v>34</v>
+      </c>
+      <c r="E35" s="18" t="str">
+        <f>C35&amp;D35</f>
+        <v>C34</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>27</v>
+      </c>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -1650,15 +1698,29 @@
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
     </row>
-    <row r="36" spans="1:18" ht="12.75">
-      <c r="A36" s="1"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="1"/>
+    <row r="36" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="17">
+        <v>2</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="18">
+        <v>35</v>
+      </c>
+      <c r="E36" s="18" t="str">
+        <f>C36&amp;D36</f>
+        <v>C35</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>21</v>
+      </c>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
@@ -1670,15 +1732,29 @@
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
     </row>
-    <row r="37" spans="1:18" ht="12.75">
-      <c r="A37" s="1"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="1"/>
+    <row r="37" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="17">
+        <v>2</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="18">
+        <v>36</v>
+      </c>
+      <c r="E37" s="18" t="str">
+        <f>C37&amp;D37</f>
+        <v>C36</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>22</v>
+      </c>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -1690,15 +1766,29 @@
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
     </row>
-    <row r="38" spans="1:18" ht="12.75">
-      <c r="A38" s="1"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="1"/>
+    <row r="38" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="17">
+        <v>2</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="18">
+        <v>37</v>
+      </c>
+      <c r="E38" s="18" t="str">
+        <f>C38&amp;D38</f>
+        <v>C37</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>9</v>
+      </c>
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
@@ -1710,17 +1800,30 @@
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
     </row>
-    <row r="39" spans="1:18" ht="12.75">
-      <c r="A39" s="1"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="1"/>
+    <row r="39" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="17">
+        <v>2</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="18">
+        <v>38</v>
+      </c>
+      <c r="E39" s="18" t="str">
+        <f>C39&amp;D39</f>
+        <v>C38</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>28</v>
+      </c>
       <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -1730,17 +1833,30 @@
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
     </row>
-    <row r="40" spans="1:18" ht="12.75">
-      <c r="A40" s="1"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="1"/>
+    <row r="40" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="17">
+        <v>2</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="18">
+        <v>39</v>
+      </c>
+      <c r="E40" s="18" t="str">
+        <f>C40&amp;D40</f>
+        <v>C39</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>19</v>
+      </c>
       <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -1750,412 +1866,130 @@
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
     </row>
-    <row r="41" spans="1:18" ht="12.75">
-      <c r="A41" s="1"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="1"/>
+    <row r="41" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="17">
+        <v>2</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="18">
+        <v>40</v>
+      </c>
+      <c r="E41" s="18" t="str">
+        <f>C41&amp;D41</f>
+        <v>C40</v>
+      </c>
+      <c r="F41" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>27</v>
+      </c>
       <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
       <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
-      <c r="P41" s="1"/>
-      <c r="Q41" s="1"/>
-      <c r="R41" s="1"/>
-    </row>
-    <row r="42" spans="1:18" ht="12.75">
-      <c r="A42" s="1"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="1"/>
+    </row>
+    <row r="42" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="17">
+        <v>2</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="18">
+        <v>41</v>
+      </c>
+      <c r="E42" s="18" t="str">
+        <f>C42&amp;D42</f>
+        <v>C41</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>21</v>
+      </c>
       <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
       <c r="K42" s="1"/>
-      <c r="L42" s="17">
+    </row>
+    <row r="43" spans="1:18" customHeight="1" ht="18.75">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="17">
+        <v>2</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="18">
+        <v>42</v>
+      </c>
+      <c r="E43" s="18" t="str">
+        <f>C43&amp;D43</f>
+        <v>C42</v>
+      </c>
+      <c r="F43" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="M42" s="18">
-        <v>3</v>
-      </c>
-      <c r="N42" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O42" s="18">
-        <v>29</v>
-      </c>
-      <c r="P42" s="18" t="str">
-        <f>N42&amp;O42</f>
-        <v>C29</v>
-      </c>
-      <c r="Q42" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="R42" s="18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:18" ht="12.75">
-      <c r="A43" s="1"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="1"/>
+      <c r="G43" s="18" t="s">
+        <v>22</v>
+      </c>
       <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
       <c r="K43" s="1"/>
-      <c r="L43" s="17">
-        <v>30</v>
-      </c>
-      <c r="M43" s="18">
-        <v>3</v>
-      </c>
-      <c r="N43" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O43" s="18">
-        <v>30</v>
-      </c>
-      <c r="P43" s="18" t="str">
-        <f>N43&amp;O43</f>
-        <v>C30</v>
-      </c>
-      <c r="Q43" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="R43" s="18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:18" ht="12.75">
+    </row>
+    <row r="44" spans="1:18" customHeight="1" ht="15">
       <c r="A44" s="1"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-      <c r="J44" s="1"/>
       <c r="K44" s="1"/>
-      <c r="L44" s="17">
-        <v>31</v>
-      </c>
-      <c r="M44" s="18">
-        <v>3</v>
-      </c>
-      <c r="N44" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O44" s="18">
-        <v>31</v>
-      </c>
-      <c r="P44" s="18" t="str">
-        <f>N44&amp;O44</f>
-        <v>C31</v>
-      </c>
-      <c r="Q44" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="R44" s="18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="45" spans="1:18" ht="12.75">
+    </row>
+    <row r="45" spans="1:18" customHeight="1" ht="15">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
       <c r="K45" s="1"/>
-      <c r="L45" s="17">
-        <v>32</v>
-      </c>
-      <c r="M45" s="18">
-        <v>3</v>
-      </c>
-      <c r="N45" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O45" s="18">
-        <v>32</v>
-      </c>
-      <c r="P45" s="18" t="str">
-        <f>N45&amp;O45</f>
-        <v>C32</v>
-      </c>
-      <c r="Q45" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="R45" s="18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" ht="12.75">
+    </row>
+    <row r="46" spans="1:18" customHeight="1" ht="15">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="J46" s="1"/>
       <c r="K46" s="1"/>
-      <c r="L46" s="17">
-        <v>33</v>
-      </c>
-      <c r="M46" s="18">
-        <v>3</v>
-      </c>
-      <c r="N46" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O46" s="18">
-        <v>33</v>
-      </c>
-      <c r="P46" s="18" t="str">
-        <f>N46&amp;O46</f>
-        <v>C33</v>
-      </c>
-      <c r="Q46" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R46" s="18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" ht="12.75">
+    </row>
+    <row r="47" spans="1:18" customHeight="1" ht="15">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
       <c r="K47" s="1"/>
-      <c r="L47" s="17">
-        <v>34</v>
-      </c>
-      <c r="M47" s="18">
-        <v>3</v>
-      </c>
-      <c r="N47" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O47" s="18">
-        <v>34</v>
-      </c>
-      <c r="P47" s="18" t="str">
-        <f>N47&amp;O47</f>
-        <v>C34</v>
-      </c>
-      <c r="Q47" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R47" s="18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="48" spans="1:18" ht="12.75">
+    </row>
+    <row r="48" spans="1:18" customHeight="1" ht="15">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
       <c r="K48" s="1"/>
-      <c r="L48" s="17">
-        <v>35</v>
-      </c>
-      <c r="M48" s="18">
-        <v>3</v>
-      </c>
-      <c r="N48" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O48" s="18">
-        <v>35</v>
-      </c>
-      <c r="P48" s="18" t="str">
-        <f>N48&amp;O48</f>
-        <v>C35</v>
-      </c>
-      <c r="Q48" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R48" s="18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="49" spans="1:18" ht="12.75">
+    </row>
+    <row r="49" spans="1:18" customHeight="1" ht="15">
       <c r="A49" s="1"/>
       <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1"/>
       <c r="K49" s="1"/>
-      <c r="L49" s="17">
-        <v>36</v>
-      </c>
-      <c r="M49" s="18">
-        <v>3</v>
-      </c>
-      <c r="N49" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O49" s="18">
-        <v>36</v>
-      </c>
-      <c r="P49" s="18" t="str">
-        <f>N49&amp;O49</f>
-        <v>C36</v>
-      </c>
-      <c r="Q49" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R49" s="18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="50" spans="1:18" ht="12.75">
+    </row>
+    <row r="50" spans="1:18" customHeight="1" ht="15">
       <c r="A50" s="1"/>
       <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1"/>
       <c r="K50" s="1"/>
-      <c r="L50" s="17">
-        <v>37</v>
-      </c>
-      <c r="M50" s="18">
-        <v>3</v>
-      </c>
-      <c r="N50" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O50" s="18">
-        <v>37</v>
-      </c>
-      <c r="P50" s="18" t="str">
-        <f>N50&amp;O50</f>
-        <v>C37</v>
-      </c>
-      <c r="Q50" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R50" s="18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="51" spans="1:18" ht="12.75">
+    </row>
+    <row r="51" spans="1:18" customHeight="1" ht="15">
       <c r="A51" s="1"/>
       <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1"/>
       <c r="K51" s="1"/>
-      <c r="L51" s="17">
-        <v>38</v>
-      </c>
-      <c r="M51" s="18">
-        <v>3</v>
-      </c>
-      <c r="N51" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O51" s="18">
-        <v>38</v>
-      </c>
-      <c r="P51" s="18" t="str">
-        <f>N51&amp;O51</f>
-        <v>C38</v>
-      </c>
-      <c r="Q51" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="R51" s="18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="52" spans="1:18" ht="12.75">
+    </row>
+    <row r="52" spans="1:18" customHeight="1" ht="15">
       <c r="A52" s="1"/>
       <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-      <c r="J52" s="1"/>
       <c r="K52" s="1"/>
-      <c r="L52" s="17">
-        <v>39</v>
-      </c>
-      <c r="M52" s="18">
-        <v>3</v>
-      </c>
-      <c r="N52" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O52" s="18">
-        <v>39</v>
-      </c>
-      <c r="P52" s="18" t="str">
-        <f>N52&amp;O52</f>
-        <v>C39</v>
-      </c>
-      <c r="Q52" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="R52" s="18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="53" spans="1:18" ht="12.75">
+    </row>
+    <row r="53" spans="1:18" customHeight="1" ht="15">
       <c r="A53" s="1"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -2167,30 +2001,8 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
-      <c r="L53" s="17">
-        <v>40</v>
-      </c>
-      <c r="M53" s="18">
-        <v>3</v>
-      </c>
-      <c r="N53" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O53" s="18">
-        <v>40</v>
-      </c>
-      <c r="P53" s="18" t="str">
-        <f>N53&amp;O53</f>
-        <v>C40</v>
-      </c>
-      <c r="Q53" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="R53" s="18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="54" spans="1:18" ht="12.75">
+    </row>
+    <row r="54" spans="1:18" customHeight="1" ht="15">
       <c r="A54" s="1"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -2202,30 +2014,8 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
-      <c r="L54" s="17">
-        <v>41</v>
-      </c>
-      <c r="M54" s="18">
-        <v>3</v>
-      </c>
-      <c r="N54" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O54" s="18">
-        <v>41</v>
-      </c>
-      <c r="P54" s="18" t="str">
-        <f>N54&amp;O54</f>
-        <v>C41</v>
-      </c>
-      <c r="Q54" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="R54" s="18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="55" spans="1:18" ht="12.75">
+    </row>
+    <row r="55" spans="1:18" customHeight="1" ht="15">
       <c r="A55" s="1"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2237,30 +2027,19 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
-      <c r="L55" s="17">
-        <v>42</v>
-      </c>
-      <c r="M55" s="18">
-        <v>3</v>
-      </c>
-      <c r="N55" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="O55" s="18">
-        <v>42</v>
-      </c>
-      <c r="P55" s="18" t="str">
-        <f>N55&amp;O55</f>
-        <v>C42</v>
-      </c>
-      <c r="Q55" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="R55" s="18" t="s">
-        <v>22</v>
-      </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>